<commit_message>
chart visualisation successful, need some changes in format to be displayed on chart
</commit_message>
<xml_diff>
--- a/output/vcp_scan_results.xlsx
+++ b/output/vcp_scan_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:Z53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,41 +563,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALB</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>193.88</v>
+        <v>360.54</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>178.76</v>
+        <v>235.38</v>
       </c>
       <c r="E2" t="n">
-        <v>146.78</v>
+        <v>226.71</v>
       </c>
       <c r="F2" t="n">
-        <v>129.48</v>
+        <v>211.38</v>
       </c>
       <c r="G2" t="n">
-        <v>192.79</v>
+        <v>324.49</v>
       </c>
       <c r="H2" t="n">
-        <v>189.34</v>
+        <v>294.96</v>
       </c>
       <c r="I2" t="n">
-        <v>180.14</v>
+        <v>255.96</v>
       </c>
       <c r="J2" t="n">
-        <v>151.57</v>
+        <v>222.07</v>
       </c>
       <c r="K2" t="n">
-        <v>141.05</v>
+        <v>211.91</v>
       </c>
       <c r="L2" t="n">
-        <v>203.56</v>
+        <v>244.02</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -605,45 +605,45 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>258.1</v>
+        <v>273</v>
       </c>
       <c r="O2" t="n">
-        <v>10.1</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>10.1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>D (Structure valid, needs tightening)</t>
         </is>
       </c>
       <c r="T2" t="n">
         <v>6</v>
       </c>
       <c r="U2" t="n">
-        <v>4.98</v>
+        <v>11</v>
       </c>
       <c r="V2" t="b">
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0.79</v>
+        <v>1.12</v>
       </c>
       <c r="X2" t="n">
-        <v>215.62</v>
+        <v>347.81</v>
       </c>
       <c r="Y2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -707,7 +707,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -717,7 +717,7 @@
         <v>4.88</v>
       </c>
       <c r="V3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W3" t="n">
         <v>0.78</v>
@@ -726,7 +726,7 @@
         <v>67.45999999999999</v>
       </c>
       <c r="Y3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z3" t="n">
         <v>1</v>
@@ -735,41 +735,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>389.08</v>
+        <v>69.12</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>369.45</v>
+        <v>62.09</v>
       </c>
       <c r="E4" t="n">
-        <v>299.69</v>
+        <v>53.88</v>
       </c>
       <c r="F4" t="n">
-        <v>268.89</v>
+        <v>51.5</v>
       </c>
       <c r="G4" t="n">
-        <v>392.69</v>
+        <v>66.7</v>
       </c>
       <c r="H4" t="n">
-        <v>387.48</v>
+        <v>64.72</v>
       </c>
       <c r="I4" t="n">
-        <v>368.03</v>
+        <v>61.83</v>
       </c>
       <c r="J4" t="n">
-        <v>310.73</v>
+        <v>55.33</v>
       </c>
       <c r="K4" t="n">
-        <v>291.4</v>
+        <v>53.12</v>
       </c>
       <c r="L4" t="n">
-        <v>134.52</v>
+        <v>65.84999999999999</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -777,85 +777,85 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>163.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="O4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>1</v>
+      </c>
+      <c r="R4" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" t="n">
         <v>6.7</v>
       </c>
-      <c r="P4" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" t="b">
-        <v>1</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>C (previous 2 of last 3 valid VCP)</t>
-        </is>
-      </c>
-      <c r="T4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" t="n">
-        <v>2.4</v>
-      </c>
       <c r="V4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>0.87</v>
+        <v>0.82</v>
       </c>
       <c r="X4" t="n">
-        <v>417.04</v>
+        <v>68.94</v>
       </c>
       <c r="Y4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BK</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>133.78</v>
+        <v>187.06</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>122.71</v>
+        <v>184.71</v>
       </c>
       <c r="E5" t="n">
-        <v>116.2</v>
+        <v>174.04</v>
       </c>
       <c r="F5" t="n">
-        <v>112.65</v>
+        <v>164.45</v>
       </c>
       <c r="G5" t="n">
-        <v>133.36</v>
+        <v>186.04</v>
       </c>
       <c r="H5" t="n">
-        <v>130.9</v>
+        <v>184.37</v>
       </c>
       <c r="I5" t="n">
-        <v>125.45</v>
+        <v>183.34</v>
       </c>
       <c r="J5" t="n">
-        <v>116.32</v>
+        <v>174.1</v>
       </c>
       <c r="K5" t="n">
-        <v>112.42</v>
+        <v>170.75</v>
       </c>
       <c r="L5" t="n">
-        <v>39.44</v>
+        <v>25.67</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -863,85 +863,85 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>68.5</v>
+        <v>60.1</v>
       </c>
       <c r="O5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="P5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="Q5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T5" t="n">
         <v>6</v>
       </c>
       <c r="U5" t="n">
-        <v>5.71</v>
+        <v>4.95</v>
       </c>
       <c r="V5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W5" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="X5" t="n">
-        <v>137.37</v>
+        <v>190.07</v>
       </c>
       <c r="Y5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Z5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHRW</t>
+          <t>BK</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>177.3</v>
+        <v>133.78</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>175.89</v>
+        <v>122.71</v>
       </c>
       <c r="E6" t="n">
-        <v>163.71</v>
+        <v>116.2</v>
       </c>
       <c r="F6" t="n">
-        <v>152.61</v>
+        <v>112.65</v>
       </c>
       <c r="G6" t="n">
-        <v>181.77</v>
+        <v>133.36</v>
       </c>
       <c r="H6" t="n">
-        <v>179.12</v>
+        <v>130.9</v>
       </c>
       <c r="I6" t="n">
-        <v>176.33</v>
+        <v>125.45</v>
       </c>
       <c r="J6" t="n">
-        <v>162.62</v>
+        <v>116.32</v>
       </c>
       <c r="K6" t="n">
-        <v>155.3</v>
+        <v>112.42</v>
       </c>
       <c r="L6" t="n">
-        <v>71.09999999999999</v>
+        <v>39.44</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -949,16 +949,16 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>106.4</v>
+        <v>68.5</v>
       </c>
       <c r="O6" t="n">
-        <v>11.3</v>
+        <v>2.6</v>
       </c>
       <c r="P6" t="n">
-        <v>11.3</v>
+        <v>2.6</v>
       </c>
       <c r="Q6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
@@ -972,62 +972,62 @@
         <v>6</v>
       </c>
       <c r="U6" t="n">
-        <v>5.18</v>
+        <v>2.82</v>
       </c>
       <c r="V6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W6" t="n">
-        <v>0.95</v>
+        <v>0.76</v>
       </c>
       <c r="X6" t="n">
-        <v>172.42</v>
+        <v>137.37</v>
       </c>
       <c r="Y6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Z6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CFG</t>
+          <t>BG</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64.42</v>
+        <v>124.61</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>60.94</v>
+        <v>123.25</v>
       </c>
       <c r="E7" t="n">
-        <v>57.67</v>
+        <v>105.99</v>
       </c>
       <c r="F7" t="n">
-        <v>55.48</v>
+        <v>99.36</v>
       </c>
       <c r="G7" t="n">
-        <v>64.29000000000001</v>
+        <v>125.24</v>
       </c>
       <c r="H7" t="n">
-        <v>63.53</v>
+        <v>124.77</v>
       </c>
       <c r="I7" t="n">
-        <v>61.97</v>
+        <v>121.92</v>
       </c>
       <c r="J7" t="n">
-        <v>57.84</v>
+        <v>109.05</v>
       </c>
       <c r="K7" t="n">
-        <v>55.91</v>
+        <v>104.8</v>
       </c>
       <c r="L7" t="n">
-        <v>49.33</v>
+        <v>34.67</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1035,13 +1035,13 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>78.3</v>
+        <v>74.5</v>
       </c>
       <c r="O7" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="P7" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="Q7" t="b">
         <v>1</v>
@@ -1058,19 +1058,19 @@
         <v>6</v>
       </c>
       <c r="U7" t="n">
-        <v>3</v>
+        <v>1.88</v>
       </c>
       <c r="V7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W7" t="n">
-        <v>1.01</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="X7" t="n">
-        <v>65.29000000000001</v>
+        <v>126.42</v>
       </c>
       <c r="Y7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Z7" t="n">
         <v>1</v>
@@ -1079,41 +1079,41 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EXPD</t>
+          <t>CHRW</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>147.23</v>
+        <v>177.3</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>145.37</v>
+        <v>175.89</v>
       </c>
       <c r="E8" t="n">
-        <v>143.63</v>
+        <v>163.71</v>
       </c>
       <c r="F8" t="n">
-        <v>137.37</v>
+        <v>152.61</v>
       </c>
       <c r="G8" t="n">
-        <v>147.75</v>
+        <v>181.77</v>
       </c>
       <c r="H8" t="n">
-        <v>147.07</v>
+        <v>179.12</v>
       </c>
       <c r="I8" t="n">
-        <v>147.02</v>
+        <v>176.33</v>
       </c>
       <c r="J8" t="n">
-        <v>142.5</v>
+        <v>162.62</v>
       </c>
       <c r="K8" t="n">
-        <v>139.44</v>
+        <v>155.3</v>
       </c>
       <c r="L8" t="n">
-        <v>6.94</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1121,13 +1121,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>40.4</v>
+        <v>106.4</v>
       </c>
       <c r="O8" t="n">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="P8" t="n">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
@@ -1137,26 +1137,26 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>A (3-step valid VCP)</t>
+          <t>B (latest 2 valid VCP)</t>
         </is>
       </c>
       <c r="T8" t="n">
         <v>6</v>
       </c>
       <c r="U8" t="n">
-        <v>2.43</v>
+        <v>5.18</v>
       </c>
       <c r="V8" t="b">
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>0.89</v>
+        <v>0.95</v>
       </c>
       <c r="X8" t="n">
-        <v>150.98</v>
+        <v>188.42</v>
       </c>
       <c r="Y8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Z8" t="n">
         <v>0</v>
@@ -1165,41 +1165,41 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50.43</v>
+        <v>122.69</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>47.95</v>
+        <v>119.58</v>
       </c>
       <c r="E9" t="n">
-        <v>46.49</v>
+        <v>96.04000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>45.53</v>
+        <v>93.64</v>
       </c>
       <c r="G9" t="n">
-        <v>50.23</v>
+        <v>123.12</v>
       </c>
       <c r="H9" t="n">
-        <v>49.61</v>
+        <v>122.9</v>
       </c>
       <c r="I9" t="n">
-        <v>48.73</v>
+        <v>117.61</v>
       </c>
       <c r="J9" t="n">
-        <v>46.79</v>
+        <v>102.5</v>
       </c>
       <c r="K9" t="n">
-        <v>45.89</v>
+        <v>98.75</v>
       </c>
       <c r="L9" t="n">
-        <v>15.73</v>
+        <v>28.66</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1207,13 +1207,13 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>44.7</v>
+        <v>62.1</v>
       </c>
       <c r="O9" t="n">
-        <v>7.6</v>
+        <v>10.8</v>
       </c>
       <c r="P9" t="n">
-        <v>7.6</v>
+        <v>10.8</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1230,16 +1230,16 @@
         <v>6</v>
       </c>
       <c r="U9" t="n">
-        <v>2.82</v>
+        <v>3.71</v>
       </c>
       <c r="V9" t="b">
         <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
       <c r="X9" t="n">
-        <v>51.1</v>
+        <v>125.59</v>
       </c>
       <c r="Y9" t="n">
         <v>7</v>
@@ -1251,41 +1251,41 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28.57</v>
+        <v>535.29</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>23.91</v>
+        <v>416.09</v>
       </c>
       <c r="E10" t="n">
-        <v>23.25</v>
+        <v>281.44</v>
       </c>
       <c r="F10" t="n">
-        <v>22.91</v>
+        <v>237.09</v>
       </c>
       <c r="G10" t="n">
-        <v>27.96</v>
+        <v>504.54</v>
       </c>
       <c r="H10" t="n">
-        <v>26.89</v>
+        <v>484.96</v>
       </c>
       <c r="I10" t="n">
-        <v>24.98</v>
+        <v>425.02</v>
       </c>
       <c r="J10" t="n">
-        <v>23.19</v>
+        <v>307.47</v>
       </c>
       <c r="K10" t="n">
-        <v>22.71</v>
+        <v>272.98</v>
       </c>
       <c r="L10" t="n">
-        <v>49.49</v>
+        <v>620.38</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1293,13 +1293,13 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>78.5</v>
+        <v>649.4</v>
       </c>
       <c r="O10" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="b">
         <v>1</v>
@@ -1316,19 +1316,19 @@
         <v>6</v>
       </c>
       <c r="U10" t="n">
-        <v>5.08</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="V10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W10" t="n">
-        <v>1.09</v>
+        <v>0.71</v>
       </c>
       <c r="X10" t="n">
-        <v>28.76</v>
+        <v>520.8</v>
       </c>
       <c r="Y10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Z10" t="n">
         <v>1</v>
@@ -1337,41 +1337,41 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IEX</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>214.93</v>
+        <v>127.44</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>199.51</v>
+        <v>117.28</v>
       </c>
       <c r="E11" t="n">
-        <v>185.85</v>
+        <v>110.77</v>
       </c>
       <c r="F11" t="n">
-        <v>180.69</v>
+        <v>106.79</v>
       </c>
       <c r="G11" t="n">
-        <v>209.83</v>
+        <v>128.11</v>
       </c>
       <c r="H11" t="n">
-        <v>205.5</v>
+        <v>126</v>
       </c>
       <c r="I11" t="n">
-        <v>200.37</v>
+        <v>120.57</v>
       </c>
       <c r="J11" t="n">
-        <v>190.78</v>
+        <v>110.87</v>
       </c>
       <c r="K11" t="n">
-        <v>188.75</v>
+        <v>106.68</v>
       </c>
       <c r="L11" t="n">
-        <v>-4.46</v>
+        <v>62.87</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1379,13 +1379,13 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>37.5</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="O11" t="n">
-        <v>1.3</v>
+        <v>4.2</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>4.2</v>
       </c>
       <c r="Q11" t="b">
         <v>1</v>
@@ -1395,23 +1395,23 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T11" t="n">
         <v>6</v>
       </c>
       <c r="U11" t="n">
-        <v>4.87</v>
+        <v>6.3</v>
       </c>
       <c r="V11" t="b">
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="X11" t="n">
-        <v>192.88</v>
+        <v>133.05</v>
       </c>
       <c r="Y11" t="n">
         <v>6</v>
@@ -1423,41 +1423,41 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>KEY</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>21.87</v>
+        <v>1867.02</v>
       </c>
       <c r="C12" t="b">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>20.7</v>
+        <v>1506.6</v>
       </c>
       <c r="E12" t="n">
-        <v>19.8</v>
+        <v>1166.63</v>
       </c>
       <c r="F12" t="n">
-        <v>19.36</v>
+        <v>1049.95</v>
       </c>
       <c r="G12" t="n">
-        <v>21.84</v>
+        <v>1752.8</v>
       </c>
       <c r="H12" t="n">
-        <v>21.56</v>
+        <v>1674.68</v>
       </c>
       <c r="I12" t="n">
-        <v>21.06</v>
+        <v>1520.46</v>
       </c>
       <c r="J12" t="n">
-        <v>19.98</v>
+        <v>1217.59</v>
       </c>
       <c r="K12" t="n">
-        <v>19.5</v>
+        <v>1115.94</v>
       </c>
       <c r="L12" t="n">
-        <v>23.56</v>
+        <v>318.85</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1465,13 +1465,13 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>52.6</v>
+        <v>347.9</v>
       </c>
       <c r="O12" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="b">
         <v>1</v>
@@ -1481,26 +1481,26 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T12" t="n">
         <v>6</v>
       </c>
       <c r="U12" t="n">
-        <v>2.52</v>
+        <v>2.7</v>
       </c>
       <c r="V12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W12" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="X12" t="n">
-        <v>22.19</v>
+        <v>1650.48</v>
       </c>
       <c r="Y12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Z12" t="n">
         <v>1</v>
@@ -1509,41 +1509,41 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MTB</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>216.44</v>
+        <v>123.19</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>212.27</v>
+        <v>122.02</v>
       </c>
       <c r="E13" t="n">
-        <v>203.44</v>
+        <v>103.01</v>
       </c>
       <c r="F13" t="n">
-        <v>200.44</v>
+        <v>100.43</v>
       </c>
       <c r="G13" t="n">
-        <v>217.24</v>
+        <v>123.68</v>
       </c>
       <c r="H13" t="n">
-        <v>216.15</v>
+        <v>123.45</v>
       </c>
       <c r="I13" t="n">
-        <v>213.91</v>
+        <v>120.14</v>
       </c>
       <c r="J13" t="n">
-        <v>206.07</v>
+        <v>108.39</v>
       </c>
       <c r="K13" t="n">
-        <v>202.47</v>
+        <v>105.54</v>
       </c>
       <c r="L13" t="n">
-        <v>1.49</v>
+        <v>11.54</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1551,13 +1551,13 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>30.5</v>
+        <v>49.4</v>
       </c>
       <c r="O13" t="n">
-        <v>8.4</v>
+        <v>7.9</v>
       </c>
       <c r="P13" t="n">
-        <v>8.4</v>
+        <v>7.9</v>
       </c>
       <c r="Q13" t="b">
         <v>0</v>
@@ -1567,26 +1567,26 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>C (previous 2 of last 3 valid VCP)</t>
+          <t>B (latest 2 valid VCP)</t>
         </is>
       </c>
       <c r="T13" t="n">
         <v>6</v>
       </c>
       <c r="U13" t="n">
-        <v>2.18</v>
+        <v>2.16</v>
       </c>
       <c r="V13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.03</v>
       </c>
       <c r="X13" t="n">
-        <v>219.7</v>
+        <v>124.37</v>
       </c>
       <c r="Y13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -1595,41 +1595,41 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>354.97</v>
+        <v>68.98</v>
       </c>
       <c r="C14" t="b">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>341.83</v>
+        <v>66.13</v>
       </c>
       <c r="E14" t="n">
-        <v>312.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>300.85</v>
+        <v>63.22</v>
       </c>
       <c r="G14" t="n">
-        <v>360.48</v>
+        <v>68.31999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>356.98</v>
+        <v>68.13</v>
       </c>
       <c r="I14" t="n">
-        <v>345.34</v>
+        <v>67.34</v>
       </c>
       <c r="J14" t="n">
-        <v>319.33</v>
+        <v>64.75</v>
       </c>
       <c r="K14" t="n">
-        <v>310.45</v>
+        <v>63.31</v>
       </c>
       <c r="L14" t="n">
-        <v>17.87</v>
+        <v>39.25</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1637,13 +1637,13 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>46.9</v>
+        <v>68.3</v>
       </c>
       <c r="O14" t="n">
-        <v>6.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="P14" t="n">
-        <v>6.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Q14" t="b">
         <v>0</v>
@@ -1653,26 +1653,26 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>A (3-step valid VCP)</t>
         </is>
       </c>
       <c r="T14" t="n">
         <v>6</v>
       </c>
       <c r="U14" t="n">
-        <v>2.98</v>
+        <v>1.51</v>
       </c>
       <c r="V14" t="b">
         <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="X14" t="n">
-        <v>378.72</v>
+        <v>71.98999999999999</v>
       </c>
       <c r="Y14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
@@ -1681,41 +1681,41 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>DOW</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>77.12</v>
+        <v>40.29</v>
       </c>
       <c r="C15" t="b">
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>76.70999999999999</v>
+        <v>36.85</v>
       </c>
       <c r="E15" t="n">
-        <v>75.06999999999999</v>
+        <v>28.6</v>
       </c>
       <c r="F15" t="n">
-        <v>71.93000000000001</v>
+        <v>27.29</v>
       </c>
       <c r="G15" t="n">
-        <v>76.78</v>
+        <v>39.18</v>
       </c>
       <c r="H15" t="n">
-        <v>76.27</v>
+        <v>38.84</v>
       </c>
       <c r="I15" t="n">
-        <v>76.42</v>
+        <v>36.72</v>
       </c>
       <c r="J15" t="n">
-        <v>74.11</v>
+        <v>31.6</v>
       </c>
       <c r="K15" t="n">
-        <v>72.29000000000001</v>
+        <v>30.96</v>
       </c>
       <c r="L15" t="n">
-        <v>0.5600000000000001</v>
+        <v>11.89</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1723,16 +1723,16 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>31.5</v>
+        <v>101.1</v>
       </c>
       <c r="O15" t="n">
-        <v>11</v>
+        <v>3.8</v>
       </c>
       <c r="P15" t="n">
-        <v>11</v>
+        <v>3.8</v>
       </c>
       <c r="Q15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" t="b">
         <v>1</v>
@@ -1746,62 +1746,62 @@
         <v>6</v>
       </c>
       <c r="U15" t="n">
-        <v>1.65</v>
+        <v>2.06</v>
       </c>
       <c r="V15" t="b">
         <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>0.8</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X15" t="n">
-        <v>78.23</v>
+        <v>38.81</v>
       </c>
       <c r="Y15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>190.17</v>
+        <v>903.5</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>171.19</v>
+        <v>776.76</v>
       </c>
       <c r="E16" t="n">
-        <v>170.03</v>
+        <v>705.24</v>
       </c>
       <c r="F16" t="n">
-        <v>163.88</v>
+        <v>683.0700000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>187.77</v>
+        <v>862.3</v>
       </c>
       <c r="H16" t="n">
-        <v>183.47</v>
+        <v>834.79</v>
       </c>
       <c r="I16" t="n">
-        <v>176.65</v>
+        <v>789.02</v>
       </c>
       <c r="J16" t="n">
-        <v>167.61</v>
+        <v>711.26</v>
       </c>
       <c r="K16" t="n">
-        <v>162.9</v>
+        <v>682.21</v>
       </c>
       <c r="L16" t="n">
-        <v>37.79</v>
+        <v>90.43000000000001</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -1809,13 +1809,13 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>66.8</v>
+        <v>119.4</v>
       </c>
       <c r="O16" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="b">
         <v>1</v>
@@ -1825,26 +1825,26 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T16" t="n">
         <v>6</v>
       </c>
       <c r="U16" t="n">
-        <v>4.52</v>
+        <v>2.65</v>
       </c>
       <c r="V16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W16" t="n">
-        <v>0.93</v>
+        <v>0.77</v>
       </c>
       <c r="X16" t="n">
-        <v>190.6</v>
+        <v>813.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Z16" t="n">
         <v>1</v>
@@ -1853,41 +1853,41 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NTRS</t>
+          <t>ETR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>164.48</v>
+        <v>116.43</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>147.52</v>
+        <v>109.39</v>
       </c>
       <c r="E17" t="n">
-        <v>139.52</v>
+        <v>99.52</v>
       </c>
       <c r="F17" t="n">
-        <v>136.3</v>
+        <v>96.53</v>
       </c>
       <c r="G17" t="n">
-        <v>164.02</v>
+        <v>114.77</v>
       </c>
       <c r="H17" t="n">
-        <v>159.47</v>
+        <v>113.6</v>
       </c>
       <c r="I17" t="n">
-        <v>151.61</v>
+        <v>109.53</v>
       </c>
       <c r="J17" t="n">
-        <v>140.59</v>
+        <v>100.72</v>
       </c>
       <c r="K17" t="n">
-        <v>136.26</v>
+        <v>97.59</v>
       </c>
       <c r="L17" t="n">
-        <v>48.6</v>
+        <v>14.47</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -1895,13 +1895,13 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>77.59999999999999</v>
+        <v>47.5</v>
       </c>
       <c r="O17" t="n">
-        <v>4.2</v>
+        <v>1.3</v>
       </c>
       <c r="P17" t="n">
-        <v>4.2</v>
+        <v>1.3</v>
       </c>
       <c r="Q17" t="b">
         <v>1</v>
@@ -1918,19 +1918,19 @@
         <v>6</v>
       </c>
       <c r="U17" t="n">
-        <v>3.83</v>
+        <v>0.67</v>
       </c>
       <c r="V17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W17" t="n">
-        <v>0.8</v>
+        <v>0.87</v>
       </c>
       <c r="X17" t="n">
-        <v>171.74</v>
+        <v>113.92</v>
       </c>
       <c r="Y17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Z17" t="n">
         <v>1</v>
@@ -1939,41 +1939,41 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RL</t>
+          <t>EXPD</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>362.21</v>
+        <v>147.23</v>
       </c>
       <c r="C18" t="b">
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>357.56</v>
+        <v>145.37</v>
       </c>
       <c r="E18" t="n">
-        <v>349.26</v>
+        <v>143.63</v>
       </c>
       <c r="F18" t="n">
-        <v>336.36</v>
+        <v>137.37</v>
       </c>
       <c r="G18" t="n">
-        <v>366.99</v>
+        <v>147.75</v>
       </c>
       <c r="H18" t="n">
-        <v>366.37</v>
+        <v>147.07</v>
       </c>
       <c r="I18" t="n">
-        <v>360.94</v>
+        <v>147.02</v>
       </c>
       <c r="J18" t="n">
-        <v>343.83</v>
+        <v>142.5</v>
       </c>
       <c r="K18" t="n">
-        <v>333.22</v>
+        <v>139.44</v>
       </c>
       <c r="L18" t="n">
-        <v>34.21</v>
+        <v>6.94</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -1981,13 +1981,13 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>63.2</v>
+        <v>40.4</v>
       </c>
       <c r="O18" t="n">
-        <v>7</v>
+        <v>10.8</v>
       </c>
       <c r="P18" t="n">
-        <v>7</v>
+        <v>10.8</v>
       </c>
       <c r="Q18" t="b">
         <v>0</v>
@@ -1997,26 +1997,26 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>A (3-step valid VCP)</t>
         </is>
       </c>
       <c r="T18" t="n">
         <v>6</v>
       </c>
       <c r="U18" t="n">
-        <v>4.1</v>
+        <v>2.43</v>
       </c>
       <c r="V18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W18" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="X18" t="n">
-        <v>389.52</v>
+        <v>150.98</v>
       </c>
       <c r="Y18" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Z18" t="n">
         <v>0</v>
@@ -2025,41 +2025,41 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>28.19</v>
+        <v>259.34</v>
       </c>
       <c r="C19" t="b">
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>27.14</v>
+        <v>212.94</v>
       </c>
       <c r="E19" t="n">
-        <v>26.6</v>
+        <v>181.82</v>
       </c>
       <c r="F19" t="n">
-        <v>26.35</v>
+        <v>181.71</v>
       </c>
       <c r="G19" t="n">
-        <v>28.15</v>
+        <v>234.19</v>
       </c>
       <c r="H19" t="n">
-        <v>27.83</v>
+        <v>222.98</v>
       </c>
       <c r="I19" t="n">
-        <v>27.48</v>
+        <v>210.17</v>
       </c>
       <c r="J19" t="n">
-        <v>26.65</v>
+        <v>188.97</v>
       </c>
       <c r="K19" t="n">
-        <v>26.16</v>
+        <v>183.02</v>
       </c>
       <c r="L19" t="n">
-        <v>14.25</v>
+        <v>101.16</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -2067,85 +2067,85 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>43.3</v>
+        <v>130.2</v>
       </c>
       <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>1</v>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>6</v>
+      </c>
+      <c r="U19" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="V19" t="b">
+        <v>1</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="X19" t="n">
+        <v>199.05</v>
+      </c>
+      <c r="Y19" t="n">
         <v>8</v>
       </c>
-      <c r="P19" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q19" t="b">
-        <v>0</v>
-      </c>
-      <c r="R19" t="b">
-        <v>1</v>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>B (latest 2 valid VCP)</t>
-        </is>
-      </c>
-      <c r="T19" t="n">
-        <v>6</v>
-      </c>
-      <c r="U19" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="V19" t="b">
-        <v>0</v>
-      </c>
-      <c r="W19" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="X19" t="n">
-        <v>28.15</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>6</v>
-      </c>
       <c r="Z19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>281.02</v>
+        <v>152.72</v>
       </c>
       <c r="C20" t="b">
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>214.64</v>
+        <v>144.32</v>
       </c>
       <c r="E20" t="n">
-        <v>192.58</v>
+        <v>139.55</v>
       </c>
       <c r="F20" t="n">
-        <v>191.52</v>
+        <v>139.05</v>
       </c>
       <c r="G20" t="n">
-        <v>262.88</v>
+        <v>152.03</v>
       </c>
       <c r="H20" t="n">
-        <v>245.52</v>
+        <v>149.75</v>
       </c>
       <c r="I20" t="n">
-        <v>223.54</v>
+        <v>145.81</v>
       </c>
       <c r="J20" t="n">
-        <v>202.54</v>
+        <v>140.1</v>
       </c>
       <c r="K20" t="n">
-        <v>198.46</v>
+        <v>137.53</v>
       </c>
       <c r="L20" t="n">
-        <v>52.61</v>
+        <v>1.82</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2153,13 +2153,13 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>84.5</v>
+        <v>30.8</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="P20" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="b">
         <v>1</v>
@@ -2169,26 +2169,26 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>B (latest 2 valid VCP)</t>
+          <t>C (previous 2 of last 3 valid VCP)</t>
         </is>
       </c>
       <c r="T20" t="n">
         <v>6</v>
       </c>
       <c r="U20" t="n">
-        <v>5.26</v>
+        <v>7.67</v>
       </c>
       <c r="V20" t="b">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>0.79</v>
+        <v>0.96</v>
       </c>
       <c r="X20" t="n">
-        <v>282.23</v>
+        <v>153.97</v>
       </c>
       <c r="Y20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Z20" t="n">
         <v>1</v>
@@ -2197,41 +2197,41 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TFC</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50.93</v>
+        <v>923.71</v>
       </c>
       <c r="C21" t="b">
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>48.17</v>
+        <v>869.99</v>
       </c>
       <c r="E21" t="n">
-        <v>47.56</v>
+        <v>855.77</v>
       </c>
       <c r="F21" t="n">
-        <v>46.65</v>
+        <v>825.5</v>
       </c>
       <c r="G21" t="n">
-        <v>50.81</v>
+        <v>920.84</v>
       </c>
       <c r="H21" t="n">
-        <v>50.04</v>
+        <v>908.29</v>
       </c>
       <c r="I21" t="n">
-        <v>49.1</v>
+        <v>888.8099999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>47.57</v>
+        <v>845.16</v>
       </c>
       <c r="K21" t="n">
-        <v>46.77</v>
+        <v>818.49</v>
       </c>
       <c r="L21" t="n">
-        <v>9.32</v>
+        <v>41.23</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2239,16 +2239,16 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>38.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="O21" t="n">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
       <c r="P21" t="n">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
       <c r="Q21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R21" t="b">
         <v>1</v>
@@ -2262,62 +2262,62 @@
         <v>6</v>
       </c>
       <c r="U21" t="n">
-        <v>2.08</v>
+        <v>4.63</v>
       </c>
       <c r="V21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W21" t="n">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="X21" t="n">
-        <v>50.48</v>
+        <v>941.74</v>
       </c>
       <c r="Y21" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Z21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>56.3</v>
+        <v>28.57</v>
       </c>
       <c r="C22" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>53.88</v>
+        <v>23.91</v>
       </c>
       <c r="E22" t="n">
-        <v>51.82</v>
+        <v>23.25</v>
       </c>
       <c r="F22" t="n">
-        <v>50.32</v>
+        <v>22.91</v>
       </c>
       <c r="G22" t="n">
-        <v>56.21</v>
+        <v>27.96</v>
       </c>
       <c r="H22" t="n">
-        <v>55.64</v>
+        <v>26.89</v>
       </c>
       <c r="I22" t="n">
-        <v>54.66</v>
+        <v>24.98</v>
       </c>
       <c r="J22" t="n">
-        <v>52.13</v>
+        <v>23.19</v>
       </c>
       <c r="K22" t="n">
-        <v>50.99</v>
+        <v>22.71</v>
       </c>
       <c r="L22" t="n">
-        <v>15.9</v>
+        <v>49.49</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
@@ -2325,16 +2325,16 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>44.9</v>
+        <v>78.5</v>
       </c>
       <c r="O22" t="n">
-        <v>6.3</v>
+        <v>0.7</v>
       </c>
       <c r="P22" t="n">
-        <v>6.3</v>
+        <v>0.7</v>
       </c>
       <c r="Q22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" t="b">
         <v>1</v>
@@ -2348,62 +2348,62 @@
         <v>6</v>
       </c>
       <c r="U22" t="n">
-        <v>2.49</v>
+        <v>2.04</v>
       </c>
       <c r="V22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W22" t="n">
-        <v>0.77</v>
+        <v>0.89</v>
       </c>
       <c r="X22" t="n">
-        <v>57</v>
+        <v>28.76</v>
       </c>
       <c r="Y22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Z22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>HLT</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>131.6</v>
+        <v>318.61</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>125.62</v>
+        <v>312.29</v>
       </c>
       <c r="E23" t="n">
-        <v>116.24</v>
+        <v>292.18</v>
       </c>
       <c r="F23" t="n">
-        <v>112.05</v>
+        <v>286.58</v>
       </c>
       <c r="G23" t="n">
-        <v>129.34</v>
+        <v>325.54</v>
       </c>
       <c r="H23" t="n">
-        <v>128.04</v>
+        <v>323.75</v>
       </c>
       <c r="I23" t="n">
-        <v>125.64</v>
+        <v>315.35</v>
       </c>
       <c r="J23" t="n">
-        <v>117.58</v>
+        <v>296.89</v>
       </c>
       <c r="K23" t="n">
-        <v>114.12</v>
+        <v>290.05</v>
       </c>
       <c r="L23" t="n">
-        <v>7.28</v>
+        <v>7.39</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -2411,16 +2411,16 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>40.5</v>
+        <v>36.4</v>
       </c>
       <c r="O23" t="n">
-        <v>1.5</v>
+        <v>7.1</v>
       </c>
       <c r="P23" t="n">
-        <v>1.5</v>
+        <v>7.1</v>
       </c>
       <c r="Q23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="b">
         <v>1</v>
@@ -2434,21 +2434,2601 @@
         <v>6</v>
       </c>
       <c r="U23" t="n">
-        <v>5.73</v>
+        <v>1.98</v>
       </c>
       <c r="V23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W23" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="X23" t="n">
+        <v>342.89</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>HST</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>21.13</v>
+      </c>
+      <c r="C24" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="E24" t="n">
+        <v>18.16</v>
+      </c>
+      <c r="F24" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="G24" t="n">
+        <v>20.94</v>
+      </c>
+      <c r="H24" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>19.88</v>
+      </c>
+      <c r="J24" t="n">
+        <v>18.48</v>
+      </c>
+      <c r="K24" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="L24" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>6</v>
+      </c>
+      <c r="U24" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="V24" t="b">
+        <v>1</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="X24" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>JBHT</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>248.73</v>
+      </c>
+      <c r="C25" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>223.8</v>
+      </c>
+      <c r="E25" t="n">
+        <v>196.99</v>
+      </c>
+      <c r="F25" t="n">
+        <v>183.18</v>
+      </c>
+      <c r="G25" t="n">
+        <v>246.89</v>
+      </c>
+      <c r="H25" t="n">
+        <v>239.75</v>
+      </c>
+      <c r="I25" t="n">
+        <v>227.12</v>
+      </c>
+      <c r="J25" t="n">
+        <v>202.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>194.85</v>
+      </c>
+      <c r="L25" t="n">
+        <v>64.72</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>93.7</v>
+      </c>
+      <c r="O25" t="n">
+        <v>2</v>
+      </c>
+      <c r="P25" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q25" t="b">
+        <v>1</v>
+      </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T25" t="n">
+        <v>6</v>
+      </c>
+      <c r="U25" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="V25" t="b">
+        <v>1</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="X25" t="n">
+        <v>253.71</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>21.87</v>
+      </c>
+      <c r="C26" t="b">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F26" t="n">
+        <v>19.36</v>
+      </c>
+      <c r="G26" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="H26" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="I26" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="J26" t="n">
+        <v>19.98</v>
+      </c>
+      <c r="K26" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="L26" t="n">
+        <v>23.56</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="O26" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="P26" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="Q26" t="b">
+        <v>1</v>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>6</v>
+      </c>
+      <c r="U26" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="V26" t="b">
+        <v>1</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="X26" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>256.72</v>
+      </c>
+      <c r="C27" t="b">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>237.08</v>
+      </c>
+      <c r="E27" t="n">
+        <v>196.84</v>
+      </c>
+      <c r="F27" t="n">
+        <v>173.94</v>
+      </c>
+      <c r="G27" t="n">
+        <v>256.92</v>
+      </c>
+      <c r="H27" t="n">
+        <v>253</v>
+      </c>
+      <c r="I27" t="n">
+        <v>239.75</v>
+      </c>
+      <c r="J27" t="n">
+        <v>200.91</v>
+      </c>
+      <c r="K27" t="n">
+        <v>185.96</v>
+      </c>
+      <c r="L27" t="n">
+        <v>231.51</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>260.5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P27" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="Q27" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T27" t="n">
+        <v>6</v>
+      </c>
+      <c r="U27" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="V27" t="b">
+        <v>1</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="X27" t="n">
+        <v>267.78</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>949.9299999999999</v>
+      </c>
+      <c r="C28" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>762.6</v>
+      </c>
+      <c r="E28" t="n">
+        <v>462.2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>379</v>
+      </c>
+      <c r="G28" t="n">
+        <v>875.98</v>
+      </c>
+      <c r="H28" t="n">
+        <v>849.36</v>
+      </c>
+      <c r="I28" t="n">
+        <v>755.5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>527.08</v>
+      </c>
+      <c r="K28" t="n">
+        <v>458.49</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1415.09</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>1444.1</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="b">
+        <v>1</v>
+      </c>
+      <c r="R28" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>D (Structure valid, needs tightening)</t>
+        </is>
+      </c>
+      <c r="T28" t="n">
+        <v>6</v>
+      </c>
+      <c r="U28" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="V28" t="b">
+        <v>1</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="X28" t="n">
+        <v>881.64</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="C29" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>70.47</v>
+      </c>
+      <c r="E29" t="n">
+        <v>54.41</v>
+      </c>
+      <c r="F29" t="n">
+        <v>53.94</v>
+      </c>
+      <c r="G29" t="n">
+        <v>72.81999999999999</v>
+      </c>
+      <c r="H29" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="I29" t="n">
+        <v>69.31999999999999</v>
+      </c>
+      <c r="J29" t="n">
+        <v>60.36</v>
+      </c>
+      <c r="K29" t="n">
+        <v>59.33</v>
+      </c>
+      <c r="L29" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="O29" t="n">
+        <v>9</v>
+      </c>
+      <c r="P29" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q29" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T29" t="n">
+        <v>6</v>
+      </c>
+      <c r="U29" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="V29" t="b">
+        <v>1</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="X29" t="n">
+        <v>72</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>354.97</v>
+      </c>
+      <c r="C30" t="b">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>341.83</v>
+      </c>
+      <c r="E30" t="n">
+        <v>312.8</v>
+      </c>
+      <c r="F30" t="n">
+        <v>300.85</v>
+      </c>
+      <c r="G30" t="n">
+        <v>360.48</v>
+      </c>
+      <c r="H30" t="n">
+        <v>356.98</v>
+      </c>
+      <c r="I30" t="n">
+        <v>345.34</v>
+      </c>
+      <c r="J30" t="n">
+        <v>319.33</v>
+      </c>
+      <c r="K30" t="n">
+        <v>310.45</v>
+      </c>
+      <c r="L30" t="n">
+        <v>17.87</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="O30" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="P30" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="Q30" t="b">
+        <v>0</v>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>A (3-step valid VCP)</t>
+        </is>
+      </c>
+      <c r="T30" t="n">
+        <v>6</v>
+      </c>
+      <c r="U30" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="V30" t="b">
+        <v>0</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="X30" t="n">
+        <v>378.72</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>542.21</v>
+      </c>
+      <c r="C31" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>425.58</v>
+      </c>
+      <c r="E31" t="n">
+        <v>326.77</v>
+      </c>
+      <c r="F31" t="n">
+        <v>276.86</v>
+      </c>
+      <c r="G31" t="n">
+        <v>500.54</v>
+      </c>
+      <c r="H31" t="n">
+        <v>472.18</v>
+      </c>
+      <c r="I31" t="n">
+        <v>431.35</v>
+      </c>
+      <c r="J31" t="n">
+        <v>341.3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>308.98</v>
+      </c>
+      <c r="L31" t="n">
+        <v>569.85</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>598.9</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="b">
+        <v>1</v>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T31" t="n">
+        <v>6</v>
+      </c>
+      <c r="U31" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="V31" t="b">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="X31" t="n">
+        <v>524.5599999999999</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>77.12</v>
+      </c>
+      <c r="C32" t="b">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="E32" t="n">
+        <v>75.06999999999999</v>
+      </c>
+      <c r="F32" t="n">
+        <v>71.93000000000001</v>
+      </c>
+      <c r="G32" t="n">
+        <v>76.78</v>
+      </c>
+      <c r="H32" t="n">
+        <v>76.27</v>
+      </c>
+      <c r="I32" t="n">
+        <v>76.42</v>
+      </c>
+      <c r="J32" t="n">
+        <v>74.11</v>
+      </c>
+      <c r="K32" t="n">
+        <v>72.29000000000001</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="O32" t="n">
+        <v>11</v>
+      </c>
+      <c r="P32" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q32" t="b">
+        <v>0</v>
+      </c>
+      <c r="R32" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T32" t="n">
+        <v>6</v>
+      </c>
+      <c r="U32" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="V32" t="b">
+        <v>1</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="X32" t="n">
+        <v>78.23</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NDSN</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>283.2</v>
+      </c>
+      <c r="C33" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>276.14</v>
+      </c>
+      <c r="E33" t="n">
+        <v>256.52</v>
+      </c>
+      <c r="F33" t="n">
+        <v>246.91</v>
+      </c>
+      <c r="G33" t="n">
+        <v>282.23</v>
+      </c>
+      <c r="H33" t="n">
+        <v>279.42</v>
+      </c>
+      <c r="I33" t="n">
+        <v>275.45</v>
+      </c>
+      <c r="J33" t="n">
+        <v>259.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>253.38</v>
+      </c>
+      <c r="L33" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="O33" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="P33" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="Q33" t="b">
+        <v>0</v>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T33" t="n">
+        <v>6</v>
+      </c>
+      <c r="U33" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="V33" t="b">
+        <v>0</v>
+      </c>
+      <c r="W33" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="X33" t="n">
+        <v>283.83</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>315.9</v>
+      </c>
+      <c r="C34" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>300.15</v>
+      </c>
+      <c r="E34" t="n">
+        <v>293.62</v>
+      </c>
+      <c r="F34" t="n">
+        <v>289.51</v>
+      </c>
+      <c r="G34" t="n">
+        <v>312.12</v>
+      </c>
+      <c r="H34" t="n">
+        <v>306.67</v>
+      </c>
+      <c r="I34" t="n">
+        <v>301</v>
+      </c>
+      <c r="J34" t="n">
+        <v>291.56</v>
+      </c>
+      <c r="K34" t="n">
+        <v>286.53</v>
+      </c>
+      <c r="L34" t="n">
+        <v>16.33</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Q34" t="b">
+        <v>1</v>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>6</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="V34" t="b">
+        <v>0</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="X34" t="n">
+        <v>321.44</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NTRS</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>164.48</v>
+      </c>
+      <c r="C35" t="b">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>147.52</v>
+      </c>
+      <c r="E35" t="n">
+        <v>139.52</v>
+      </c>
+      <c r="F35" t="n">
+        <v>136.3</v>
+      </c>
+      <c r="G35" t="n">
+        <v>164.02</v>
+      </c>
+      <c r="H35" t="n">
+        <v>159.47</v>
+      </c>
+      <c r="I35" t="n">
+        <v>151.61</v>
+      </c>
+      <c r="J35" t="n">
+        <v>140.59</v>
+      </c>
+      <c r="K35" t="n">
+        <v>136.26</v>
+      </c>
+      <c r="L35" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="O35" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="P35" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q35" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T35" t="n">
+        <v>6</v>
+      </c>
+      <c r="U35" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="V35" t="b">
+        <v>0</v>
+      </c>
+      <c r="W35" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="X35" t="n">
+        <v>171.74</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>205.81</v>
+      </c>
+      <c r="C36" t="b">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>201.11</v>
+      </c>
+      <c r="E36" t="n">
+        <v>170.63</v>
+      </c>
+      <c r="F36" t="n">
+        <v>165.51</v>
+      </c>
+      <c r="G36" t="n">
+        <v>214.01</v>
+      </c>
+      <c r="H36" t="n">
+        <v>211.39</v>
+      </c>
+      <c r="I36" t="n">
+        <v>201.74</v>
+      </c>
+      <c r="J36" t="n">
+        <v>181.8</v>
+      </c>
+      <c r="K36" t="n">
+        <v>177.86</v>
+      </c>
+      <c r="L36" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="O36" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="P36" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="Q36" t="b">
+        <v>0</v>
+      </c>
+      <c r="R36" t="b">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T36" t="n">
+        <v>6</v>
+      </c>
+      <c r="U36" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="V36" t="b">
+        <v>1</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="X36" t="n">
+        <v>224.42</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>103.03</v>
+      </c>
+      <c r="C37" t="b">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>70.53</v>
+      </c>
+      <c r="E37" t="n">
+        <v>60.32</v>
+      </c>
+      <c r="F37" t="n">
+        <v>58.17</v>
+      </c>
+      <c r="G37" t="n">
+        <v>94.38</v>
+      </c>
+      <c r="H37" t="n">
+        <v>86.23</v>
+      </c>
+      <c r="I37" t="n">
+        <v>75.01000000000001</v>
+      </c>
+      <c r="J37" t="n">
+        <v>64.03</v>
+      </c>
+      <c r="K37" t="n">
+        <v>61.99</v>
+      </c>
+      <c r="L37" t="n">
+        <v>131.16</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>168.2</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="b">
+        <v>1</v>
+      </c>
+      <c r="R37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>D (Structure valid, needs tightening)</t>
+        </is>
+      </c>
+      <c r="T37" t="n">
+        <v>6</v>
+      </c>
+      <c r="U37" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="V37" t="b">
+        <v>1</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="X37" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PNC</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>220.71</v>
+      </c>
+      <c r="C38" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>212.98</v>
+      </c>
+      <c r="E38" t="n">
+        <v>204.96</v>
+      </c>
+      <c r="F38" t="n">
+        <v>202.02</v>
+      </c>
+      <c r="G38" t="n">
+        <v>221.46</v>
+      </c>
+      <c r="H38" t="n">
+        <v>219.65</v>
+      </c>
+      <c r="I38" t="n">
+        <v>216.14</v>
+      </c>
+      <c r="J38" t="n">
+        <v>207.33</v>
+      </c>
+      <c r="K38" t="n">
+        <v>203.39</v>
+      </c>
+      <c r="L38" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="O38" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="P38" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="Q38" t="b">
+        <v>0</v>
+      </c>
+      <c r="R38" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T38" t="n">
+        <v>6</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="V38" t="b">
+        <v>0</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="X38" t="n">
+        <v>228.05</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>141.41</v>
+      </c>
+      <c r="C39" t="b">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>136.53</v>
+      </c>
+      <c r="E39" t="n">
+        <v>129.09</v>
+      </c>
+      <c r="F39" t="n">
+        <v>123.71</v>
+      </c>
+      <c r="G39" t="n">
+        <v>140.96</v>
+      </c>
+      <c r="H39" t="n">
+        <v>139.63</v>
+      </c>
+      <c r="I39" t="n">
+        <v>136.74</v>
+      </c>
+      <c r="J39" t="n">
+        <v>129.29</v>
+      </c>
+      <c r="K39" t="n">
+        <v>126.47</v>
+      </c>
+      <c r="L39" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>42</v>
+      </c>
+      <c r="O39" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P39" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q39" t="b">
+        <v>1</v>
+      </c>
+      <c r="R39" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T39" t="n">
+        <v>6</v>
+      </c>
+      <c r="U39" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="V39" t="b">
+        <v>0</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="X39" t="n">
+        <v>145.1</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>362.21</v>
+      </c>
+      <c r="C40" t="b">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>357.56</v>
+      </c>
+      <c r="E40" t="n">
+        <v>349.26</v>
+      </c>
+      <c r="F40" t="n">
+        <v>336.36</v>
+      </c>
+      <c r="G40" t="n">
+        <v>366.99</v>
+      </c>
+      <c r="H40" t="n">
+        <v>366.37</v>
+      </c>
+      <c r="I40" t="n">
+        <v>360.94</v>
+      </c>
+      <c r="J40" t="n">
+        <v>343.83</v>
+      </c>
+      <c r="K40" t="n">
+        <v>333.22</v>
+      </c>
+      <c r="L40" t="n">
+        <v>34.21</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="O40" t="n">
+        <v>7</v>
+      </c>
+      <c r="P40" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q40" t="b">
+        <v>0</v>
+      </c>
+      <c r="R40" t="b">
+        <v>1</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>6</v>
+      </c>
+      <c r="U40" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="V40" t="b">
+        <v>0</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="X40" t="n">
+        <v>389.52</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="C41" t="b">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>27.14</v>
+      </c>
+      <c r="E41" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F41" t="n">
+        <v>26.35</v>
+      </c>
+      <c r="G41" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="H41" t="n">
+        <v>27.83</v>
+      </c>
+      <c r="I41" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="J41" t="n">
+        <v>26.65</v>
+      </c>
+      <c r="K41" t="n">
+        <v>26.16</v>
+      </c>
+      <c r="L41" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="O41" t="n">
+        <v>8</v>
+      </c>
+      <c r="P41" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q41" t="b">
+        <v>0</v>
+      </c>
+      <c r="R41" t="b">
+        <v>1</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T41" t="n">
+        <v>6</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="V41" t="b">
+        <v>1</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="X41" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>56.92</v>
+      </c>
+      <c r="C42" t="b">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>50.82</v>
+      </c>
+      <c r="E42" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="F42" t="n">
+        <v>41.07</v>
+      </c>
+      <c r="G42" t="n">
+        <v>55.23</v>
+      </c>
+      <c r="H42" t="n">
+        <v>53.81</v>
+      </c>
+      <c r="I42" t="n">
+        <v>51.26</v>
+      </c>
+      <c r="J42" t="n">
+        <v>45.58</v>
+      </c>
+      <c r="K42" t="n">
+        <v>44.03</v>
+      </c>
+      <c r="L42" t="n">
+        <v>44.84</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="b">
+        <v>1</v>
+      </c>
+      <c r="R42" t="b">
+        <v>1</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T42" t="n">
+        <v>6</v>
+      </c>
+      <c r="U42" t="n">
+        <v>2</v>
+      </c>
+      <c r="V42" t="b">
+        <v>1</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="X42" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SWK</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>78.53</v>
+      </c>
+      <c r="C43" t="b">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="E43" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="F43" t="n">
+        <v>73.45999999999999</v>
+      </c>
+      <c r="G43" t="n">
+        <v>76.56999999999999</v>
+      </c>
+      <c r="H43" t="n">
+        <v>75.01000000000001</v>
+      </c>
+      <c r="I43" t="n">
+        <v>74.97</v>
+      </c>
+      <c r="J43" t="n">
+        <v>74.69</v>
+      </c>
+      <c r="K43" t="n">
+        <v>74.47</v>
+      </c>
+      <c r="L43" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="O43" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="P43" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="Q43" t="b">
+        <v>0</v>
+      </c>
+      <c r="R43" t="b">
+        <v>1</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T43" t="n">
+        <v>6</v>
+      </c>
+      <c r="U43" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="V43" t="b">
+        <v>0</v>
+      </c>
+      <c r="W43" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="X43" t="n">
+        <v>79.86</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="C44" t="b">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>96.84</v>
+      </c>
+      <c r="E44" t="n">
+        <v>90.06</v>
+      </c>
+      <c r="F44" t="n">
+        <v>89.38</v>
+      </c>
+      <c r="G44" t="n">
+        <v>101.46</v>
+      </c>
+      <c r="H44" t="n">
+        <v>99.37</v>
+      </c>
+      <c r="I44" t="n">
+        <v>96.83</v>
+      </c>
+      <c r="J44" t="n">
+        <v>92.59999999999999</v>
+      </c>
+      <c r="K44" t="n">
+        <v>91.58</v>
+      </c>
+      <c r="L44" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="b">
+        <v>1</v>
+      </c>
+      <c r="R44" t="b">
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>A (3-step valid VCP)</t>
+        </is>
+      </c>
+      <c r="T44" t="n">
+        <v>6</v>
+      </c>
+      <c r="U44" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="V44" t="b">
+        <v>1</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="X44" t="n">
+        <v>99.54000000000001</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>152</v>
+      </c>
+      <c r="C45" t="b">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>132.79</v>
+      </c>
+      <c r="E45" t="n">
+        <v>125.47</v>
+      </c>
+      <c r="F45" t="n">
+        <v>121.55</v>
+      </c>
+      <c r="G45" t="n">
+        <v>150.33</v>
+      </c>
+      <c r="H45" t="n">
+        <v>145.57</v>
+      </c>
+      <c r="I45" t="n">
+        <v>137.11</v>
+      </c>
+      <c r="J45" t="n">
+        <v>126.17</v>
+      </c>
+      <c r="K45" t="n">
+        <v>122.14</v>
+      </c>
+      <c r="L45" t="n">
+        <v>47.09</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="O45" t="n">
         <v>1.3</v>
       </c>
-      <c r="X23" t="n">
-        <v>132.03</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>6</v>
-      </c>
-      <c r="Z23" t="n">
+      <c r="P45" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Q45" t="b">
+        <v>1</v>
+      </c>
+      <c r="R45" t="b">
+        <v>1</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T45" t="n">
+        <v>6</v>
+      </c>
+      <c r="U45" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="V45" t="b">
+        <v>1</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="X45" t="n">
+        <v>154.02</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>229.27</v>
+      </c>
+      <c r="C46" t="b">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>191.29</v>
+      </c>
+      <c r="E46" t="n">
+        <v>174</v>
+      </c>
+      <c r="F46" t="n">
+        <v>162.77</v>
+      </c>
+      <c r="G46" t="n">
+        <v>221.51</v>
+      </c>
+      <c r="H46" t="n">
+        <v>211.08</v>
+      </c>
+      <c r="I46" t="n">
+        <v>196.59</v>
+      </c>
+      <c r="J46" t="n">
+        <v>176.33</v>
+      </c>
+      <c r="K46" t="n">
+        <v>169.55</v>
+      </c>
+      <c r="L46" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>90.7</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="b">
+        <v>1</v>
+      </c>
+      <c r="R46" t="b">
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T46" t="n">
+        <v>6</v>
+      </c>
+      <c r="U46" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="V46" t="b">
+        <v>1</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="X46" t="n">
+        <v>227.46</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>TRGP</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>254.28</v>
+      </c>
+      <c r="C47" t="b">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>239.77</v>
+      </c>
+      <c r="E47" t="n">
+        <v>197.47</v>
+      </c>
+      <c r="F47" t="n">
+        <v>188.69</v>
+      </c>
+      <c r="G47" t="n">
+        <v>246.44</v>
+      </c>
+      <c r="H47" t="n">
+        <v>243.3</v>
+      </c>
+      <c r="I47" t="n">
+        <v>235.19</v>
+      </c>
+      <c r="J47" t="n">
+        <v>208.69</v>
+      </c>
+      <c r="K47" t="n">
+        <v>201.02</v>
+      </c>
+      <c r="L47" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Q47" t="b">
+        <v>1</v>
+      </c>
+      <c r="R47" t="b">
+        <v>1</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T47" t="n">
+        <v>6</v>
+      </c>
+      <c r="U47" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="V47" t="b">
+        <v>1</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="X47" t="n">
+        <v>249.73</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TXT</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>94.72</v>
+      </c>
+      <c r="C48" t="b">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>92.15000000000001</v>
+      </c>
+      <c r="E48" t="n">
+        <v>88.62</v>
+      </c>
+      <c r="F48" t="n">
+        <v>86.67</v>
+      </c>
+      <c r="G48" t="n">
+        <v>91.45999999999999</v>
+      </c>
+      <c r="H48" t="n">
+        <v>90.97</v>
+      </c>
+      <c r="I48" t="n">
+        <v>91.23999999999999</v>
+      </c>
+      <c r="J48" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="K48" t="n">
+        <v>87.59</v>
+      </c>
+      <c r="L48" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="O48" t="n">
+        <v>6</v>
+      </c>
+      <c r="P48" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q48" t="b">
+        <v>0</v>
+      </c>
+      <c r="R48" t="b">
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T48" t="n">
+        <v>6</v>
+      </c>
+      <c r="U48" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="V48" t="b">
+        <v>1</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="X48" t="n">
+        <v>93.11</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TFC</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>50.93</v>
+      </c>
+      <c r="C49" t="b">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="E49" t="n">
+        <v>47.56</v>
+      </c>
+      <c r="F49" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="G49" t="n">
+        <v>50.81</v>
+      </c>
+      <c r="H49" t="n">
+        <v>50.04</v>
+      </c>
+      <c r="I49" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>47.57</v>
+      </c>
+      <c r="K49" t="n">
+        <v>46.77</v>
+      </c>
+      <c r="L49" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="O49" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P49" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q49" t="b">
+        <v>0</v>
+      </c>
+      <c r="R49" t="b">
+        <v>1</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T49" t="n">
+        <v>6</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="V49" t="b">
+        <v>1</v>
+      </c>
+      <c r="W49" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="X49" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>107.57</v>
+      </c>
+      <c r="C50" t="b">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>103.66</v>
+      </c>
+      <c r="E50" t="n">
+        <v>99.19</v>
+      </c>
+      <c r="F50" t="n">
+        <v>95.64</v>
+      </c>
+      <c r="G50" t="n">
+        <v>106.47</v>
+      </c>
+      <c r="H50" t="n">
+        <v>104.96</v>
+      </c>
+      <c r="I50" t="n">
+        <v>103.96</v>
+      </c>
+      <c r="J50" t="n">
+        <v>101.08</v>
+      </c>
+      <c r="K50" t="n">
+        <v>100.59</v>
+      </c>
+      <c r="L50" t="n">
+        <v>-7.53</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="O50" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="P50" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="Q50" t="b">
+        <v>0</v>
+      </c>
+      <c r="R50" t="b">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>B (latest 2 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T50" t="n">
+        <v>6</v>
+      </c>
+      <c r="U50" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="V50" t="b">
+        <v>1</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="X50" t="n">
+        <v>98.38</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="C51" t="b">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E51" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="F51" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="G51" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="H51" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="I51" t="n">
+        <v>14.09</v>
+      </c>
+      <c r="J51" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="K51" t="n">
+        <v>12.33</v>
+      </c>
+      <c r="L51" t="n">
+        <v>56.83</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="O51" t="n">
+        <v>6</v>
+      </c>
+      <c r="P51" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q51" t="b">
+        <v>0</v>
+      </c>
+      <c r="R51" t="b">
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T51" t="n">
+        <v>6</v>
+      </c>
+      <c r="U51" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="V51" t="b">
+        <v>0</v>
+      </c>
+      <c r="W51" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="X51" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>WAB</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>264.95</v>
+      </c>
+      <c r="C52" t="b">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>255.33</v>
+      </c>
+      <c r="E52" t="n">
+        <v>228.31</v>
+      </c>
+      <c r="F52" t="n">
+        <v>219.58</v>
+      </c>
+      <c r="G52" t="n">
+        <v>264.63</v>
+      </c>
+      <c r="H52" t="n">
+        <v>262.03</v>
+      </c>
+      <c r="I52" t="n">
+        <v>254.59</v>
+      </c>
+      <c r="J52" t="n">
+        <v>234.39</v>
+      </c>
+      <c r="K52" t="n">
+        <v>227.57</v>
+      </c>
+      <c r="L52" t="n">
+        <v>13.44</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="O52" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P52" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Q52" t="b">
+        <v>1</v>
+      </c>
+      <c r="R52" t="b">
+        <v>1</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T52" t="n">
+        <v>6</v>
+      </c>
+      <c r="U52" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="V52" t="b">
+        <v>0</v>
+      </c>
+      <c r="W52" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="X52" t="n">
+        <v>269.45</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>WELL</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>216.91</v>
+      </c>
+      <c r="C53" t="b">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>206.09</v>
+      </c>
+      <c r="E53" t="n">
+        <v>193.52</v>
+      </c>
+      <c r="F53" t="n">
+        <v>186.25</v>
+      </c>
+      <c r="G53" t="n">
+        <v>211.99</v>
+      </c>
+      <c r="H53" t="n">
+        <v>209.36</v>
+      </c>
+      <c r="I53" t="n">
+        <v>205.16</v>
+      </c>
+      <c r="J53" t="n">
+        <v>192.82</v>
+      </c>
+      <c r="K53" t="n">
+        <v>186.87</v>
+      </c>
+      <c r="L53" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q53" t="b">
+        <v>1</v>
+      </c>
+      <c r="R53" t="b">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>C (previous 2 of last 3 valid VCP)</t>
+        </is>
+      </c>
+      <c r="T53" t="n">
+        <v>6</v>
+      </c>
+      <c r="U53" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="V53" t="b">
+        <v>0</v>
+      </c>
+      <c r="W53" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="X53" t="n">
+        <v>214.51</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z53" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>